<commit_message>
docs(reports): migrate source templates to ExcelForge
</commit_message>
<xml_diff>
--- a/students-courses/share/documents/courses/reports/course-participants.xlsx
+++ b/students-courses/share/documents/courses/reports/course-participants.xlsx
@@ -82,17 +82,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
-      <color theme="1"/>
-      <family val="2"/>
-      <scheme val="minor"/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
@@ -163,7 +161,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyNumberFormat="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -179,16 +177,6 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
@@ -513,121 +501,116 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <sheetPr>
-    <pageSetUpPr fitToPage="1"/>
-  </sheetPr>
-  <dimension ref="A1:F10"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <cols>
-    <col min="1" max="1" width="9" hidden="1" customWidth="1"/>
+    <col min="1" max="1" width="9" customWidth="1" hidden="1"/>
     <col min="2" max="2" width="7" customWidth="1"/>
     <col min="3" max="3" width="18" customWidth="1"/>
     <col min="4" max="4" width="34" customWidth="1"/>
     <col min="5" max="5" width="32" customWidth="1"/>
-    <col min="6" max="6" width="9" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="9" customWidth="1" hidden="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B1" s="1" t="s">
+    <row r="1" ht="30" customHeight="1">
+      <c r="B1" t="s" s="1">
         <v>0</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="E1" s="1"/>
     </row>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B2" s="2" t="s">
+    <row r="2">
+      <c r="B2" t="s" s="2">
         <v>1</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" t="s" s="3">
         <v>2</v>
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
+    <row r="3">
+      <c r="B3" t="s" s="2">
         <v>3</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" t="s" s="3">
         <v>4</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" ht="42" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
+    <row r="4" ht="42" customHeight="1">
+      <c r="B4" t="s" s="2">
         <v>5</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" t="s" s="4">
         <v>6</v>
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B5" s="2" t="s">
+    <row r="5">
+      <c r="B5" t="s" s="2">
         <v>7</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" t="s" s="5">
         <v>8</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" t="s" s="2">
         <v>9</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" t="s" s="5">
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="6">
       <c r="B6" s="6"/>
       <c r="C6" s="6"/>
       <c r="D6" s="6"/>
       <c r="E6" s="6"/>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="7">
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
       <c r="D7" s="6"/>
       <c r="E7" s="6"/>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="7" t="s">
+    <row r="8">
+      <c r="B8" t="s" s="7">
         <v>11</v>
       </c>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B9" s="8" t="s">
+    <row r="9">
+      <c r="B9" t="s" s="8">
         <v>12</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" t="s" s="8">
         <v>13</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" t="s" s="8">
         <v>3</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="E9" t="s" s="8">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="10">
       <c r="A10" t="s">
         <v>15</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" t="s" s="3">
         <v>16</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" t="s" s="3">
         <v>17</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="D10" t="s" s="3">
         <v>18</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="E10" t="s" s="3">
         <v>19</v>
       </c>
       <c r="F10" t="s">
@@ -643,6 +626,6 @@
     <mergeCell ref="B8:E8"/>
   </mergeCells>
   <pageMargins left="0.35" right="0.35" top="0.5" bottom="0.5" header="0.2" footer="0.2"/>
-  <pageSetup orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0" scale="100" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>